<commit_message>
Update SMD component sizes
</commit_message>
<xml_diff>
--- a/phantom-injector-hat-BOM.xlsx
+++ b/phantom-injector-hat-BOM.xlsx
@@ -449,11 +449,11 @@
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>--- Boost converter (LT8362 reference design) ---</t>
+          <t>--- Boost converter (LT8362 reference design, hand-assembly sizing) ---</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LT8362EMSE#PBF</t>
+          <t>LT8362HMSE#PBF</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Boost converter, 60V SW, 400 kHz SSFM</t>
+          <t>Boost converter, 60V SW, 400 kHz SSFM, H-grade (-40~125°C)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -574,16 +574,16 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>LT8362EMSE#PBF</t>
+          <t>LT8362HMSE#PBF</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>LT8362EMSE#PBF-ND</t>
+          <t>LT8362HMSE#PBF-ND</t>
         </is>
       </c>
       <c r="I3" s="3" t="n">
-        <v>6.36</v>
+        <v>6.95</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -595,10 +595,10 @@
         <v>6</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>6.36</v>
+        <v>6.95</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>38.16</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="4">
@@ -619,12 +619,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shielded power inductor, ≥500 mA Isat</t>
+          <t>Shielded power inductor, ≥1.4A Isat</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5.3×5.5 mm</t>
+          <t>5.3×5.5 mm SMT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7.3×7.3 mm</t>
+          <t>7.3×7.3 mm SMT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -734,17 +734,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DFLS260</t>
+          <t>B260A</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>60V 2A Schottky, low VF</t>
+          <t>60V 2A Schottky in SMA package (easier hand assembly)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SOD-123FL</t>
+          <t>SMA / DO-214AC</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -754,16 +754,16 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DFLS260-7</t>
+          <t>B260A-13-F</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>DFLS260-7DICT-ND</t>
+          <t>B260A-FDICT-ND</t>
         </is>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.46</v>
+        <v>0.65</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
@@ -775,10 +775,10 @@
         <v>6</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.46</v>
+        <v>0.65</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>2.76</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>742792040</t>
+          <t>742792044</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>732-742792040-ND</t>
+          <t>732-742792044-ND</t>
         </is>
       </c>
       <c r="I7" s="3" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -874,12 +874,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>RC0603FR-071ML</t>
+          <t>RC0805FR-071ML</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>YAG2070CT-ND</t>
+          <t>311-1.0MCRCT-ND</t>
         </is>
       </c>
       <c r="I8" s="3" t="n">
@@ -924,7 +924,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>RC0603FR-0734K8L</t>
+          <t>RC0805FR-0734K8L</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>311-34.8KHRCT-ND</t>
+          <t>311-34.8KCRCT-ND</t>
         </is>
       </c>
       <c r="I9" s="3" t="n">
@@ -984,7 +984,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>RC0603FR-07121KL</t>
+          <t>RC0805FR-07121KL</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>311-121KHRCT-ND</t>
+          <t>311-121KCRCT-ND</t>
         </is>
       </c>
       <c r="I10" s="3" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1054,12 +1054,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>RC0603FR-0722K1L</t>
+          <t>RC0805FR-0722K1L</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>311-22.1KHRCT-ND</t>
+          <t>311-22.1KCRCT-ND</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1114,12 +1114,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0805FR-07100KL</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>311-100KHRCT-ND</t>
+          <t>311-100KCRCT-ND</t>
         </is>
       </c>
       <c r="I12" s="3" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1174,16 +1174,16 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>GRM31CR71H106KA12L</t>
+          <t>GRM32ER71H106KA12L</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>490-7327-1-ND</t>
+          <t>490-10758-1-ND</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0.55</v>
+        <v>0.95</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -1195,10 +1195,10 @@
         <v>6</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.55</v>
+        <v>0.95</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>3.3</v>
+        <v>5.699999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1234,16 +1234,16 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>GRM188R71E105KA12D</t>
+          <t>GRM21BR71E105KA99L</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>490-3895-1-ND</t>
+          <t>490-3334-1-ND</t>
         </is>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
@@ -1255,10 +1255,10 @@
         <v>6</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.8400000000000001</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="15">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1294,16 +1294,16 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>GRM21BR72A105KA01L</t>
+          <t>GRM31CR72A105KA01L</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>490-7331-1-ND</t>
+          <t>490-5524-1-ND</t>
         </is>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0.5</v>
+        <v>0.65</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
@@ -1315,10 +1315,10 @@
         <v>6</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>0.5</v>
+        <v>0.65</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="16">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1354,16 +1354,16 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>GRM188R71H102KA01D</t>
+          <t>GRM21BR71H102KA01L</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>490-3258-1-ND</t>
+          <t>490-3326-1-ND</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="J16" t="n">
         <v>1</v>
@@ -1375,10 +1375,10 @@
         <v>6</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="17">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1414,16 +1414,16 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>GRM188R71H103KA01D</t>
+          <t>GRM21BR71H103KA01L</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>490-1497-1-ND</t>
+          <t>490-1666-1-ND</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="J17" t="n">
         <v>1</v>
@@ -1435,10 +1435,10 @@
         <v>6</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="18">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1534,16 +1534,16 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>GRM188R72A104KA35D</t>
+          <t>GRM21BR72A104KA01L</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>490-10765-1-ND</t>
+          <t>490-7297-1-ND</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -1555,10 +1555,10 @@
         <v>6</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>1.2</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="20">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1594,16 +1594,16 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>GRM31CR71H475KA12L</t>
+          <t>GRM32ER71H475KA88L</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>490-7333-1-ND</t>
+          <t>490-7359-1-ND</t>
         </is>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
@@ -1615,10 +1615,10 @@
         <v>6</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="21">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1714,16 +1714,16 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>GRM188R72A104KA35D</t>
+          <t>GRM21BR72A104KA01L</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>490-10765-1-ND</t>
+          <t>490-7297-1-ND</t>
         </is>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
@@ -1735,10 +1735,10 @@
         <v>6</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>1.2</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="23">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1774,16 +1774,16 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>GRM188R72A104KA35D</t>
+          <t>GRM21BR72A104KA01L</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>490-10765-1-ND</t>
+          <t>490-7297-1-ND</t>
         </is>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
@@ -1795,10 +1795,10 @@
         <v>6</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>1.2</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="24">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4.7 pF C0G</t>
+          <t>4.7 pF C0G 50V</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1834,16 +1834,16 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>GRM1885C1H4R7CA01D</t>
+          <t>GRM2165C1H4R7CA01D</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>490-1393-1-ND</t>
+          <t>490-3303-1-ND</t>
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
@@ -1855,10 +1855,10 @@
         <v>6</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.6000000000000001</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="25">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>P48 enable, L channel, right-angle PCB</t>
+          <t>P48 enable, L channel, right-angle PCB-mount</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>P48 enable, R channel, right-angle PCB</t>
+          <t>P48 enable, R channel, right-angle PCB-mount</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2471,7 +2471,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>--- Connectors and indicators ---</t>
+          <t>--- Connectors and indicators (all through-hole) ---</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2498,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2.54 mm pitch</t>
+          <t>THT 2.54 mm pitch</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2548,17 +2548,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2×3 box header</t>
+          <t>2×3 box header polarized</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>To HiFiBerry J4 ribbon, polarized</t>
+          <t>To HiFiBerry J4 ribbon</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2.54 mm pitch</t>
+          <t>THT 2.54 mm pitch</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2.54 mm pitch</t>
+          <t>THT 2.54 mm pitch</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2.54 mm pitch</t>
+          <t>THT 2.54 mm pitch</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>T-1</t>
+          <t>THT T-1</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2842,10 +2842,10 @@
         </is>
       </c>
       <c r="M43" s="5" t="n">
-        <v>33.23</v>
+        <v>34.87999999999999</v>
       </c>
       <c r="N43" s="5" t="n">
-        <v>199.38</v>
+        <v>209.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>